<commit_message>
fix the D sector disaggregation to be more precise in the mappings
</commit_message>
<xml_diff>
--- a/source-data/mappings/eurostat-io-industry-to-fingreen-industry-map.xlsx
+++ b/source-data/mappings/eurostat-io-industry-to-fingreen-industry-map.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="ava" sheetId="1" state="visible" r:id="rId3"/>
@@ -1145,7 +1145,7 @@
         <v>45</v>
       </c>
       <c r="D26" s="7" t="n">
-        <v>0.937</v>
+        <v>0.936513719564738</v>
       </c>
       <c r="E26" s="5" t="s">
         <v>11</v>
@@ -1163,7 +1163,7 @@
         <v>45</v>
       </c>
       <c r="D27" s="7" t="n">
-        <v>0.021</v>
+        <v>0.0206205834596813</v>
       </c>
       <c r="E27" s="5" t="s">
         <v>11</v>
@@ -1181,7 +1181,7 @@
         <v>45</v>
       </c>
       <c r="D28" s="7" t="n">
-        <v>0.043</v>
+        <v>0.0428656969755808</v>
       </c>
       <c r="E28" s="5" t="s">
         <v>11</v>
@@ -2358,7 +2358,7 @@
         <v>45</v>
       </c>
       <c r="D26" s="1" t="n">
-        <v>0.937</v>
+        <v>0.936513719564738</v>
       </c>
       <c r="E26" s="5" t="s">
         <v>11</v>
@@ -2375,7 +2375,7 @@
         <v>45</v>
       </c>
       <c r="D27" s="1" t="n">
-        <v>0.021</v>
+        <v>0.0206205834596813</v>
       </c>
       <c r="E27" s="5" t="s">
         <v>11</v>
@@ -2392,7 +2392,7 @@
         <v>45</v>
       </c>
       <c r="D28" s="1" t="n">
-        <v>0.043</v>
+        <v>0.0428656969755808</v>
       </c>
       <c r="E28" s="5" t="s">
         <v>11</v>

</xml_diff>